<commit_message>
Financeiro: adiciona 2024 na Metalurgia (24) e corrige comparação de ano
Dados_Financeiros_Metalurgia_24.csv ganhou a linha de 2024 (Fundição
24.5 segue em 2023 — fonte não atualizou esse recorte ainda). Corrige
a análise de produtividade em Estudos Especiais, que comparava o
último ano de cada série independentemente e passou a cruzar anos
diferentes (Fundição 2023 x Metalurgia 2024) — agora busca o ano da
Metalurgia que bate com o último ano disponível da Fundição.
</commit_message>
<xml_diff>
--- a/data/downloads/Financeiro.xlsx
+++ b/data/downloads/Financeiro.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1190,8 +1190,46 @@
         <v>110445050</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2610</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>256862</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>448110326</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>32685166</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>19799994</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>435393205</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>419436237</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>286951084</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>229182649</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>424962011</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>138010927</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Fonte: IBGE/PIA-Empresa, 2007-2023.</t>
         </is>
@@ -1199,7 +1237,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Financeiro: adiciona 2024 na Fundição (24.5), atualiza notas pra 2007–2024
Fundição agora cobre o mesmo período que Metalurgia (24). Gráfico de
participação da Fundição na Metalurgia passa a ter ponto real em 2024
(antes ficava em branco por falta desse dado); análise de
produtividade em Estudos Especiais passa a comparar 2024 com 2024.
</commit_message>
<xml_diff>
--- a/data/downloads/Financeiro.xlsx
+++ b/data/downloads/Financeiro.xlsx
@@ -1249,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1981,8 +1981,46 @@
         <v>5394416</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>766</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>31682</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1749906</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>790616</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>12346918</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>12129822</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>11359870</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>7147665</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>5942477</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>12482713</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>5335048</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Reúne 2451+2452 sem abertura entre eles. Fonte: IBGE/PIA-Empresa, 2007-2023.</t>
         </is>
@@ -1990,7 +2028,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Comtrade atualizado (cesta HS certa, sem duplicação) e financeiro por classe (2024)
Comtrade_Global_Fundicao_2451/2452.csv: cesta de HS agora alinhada com
o Comex Stat (7325 pro 2451; 6 metais pro 2452, mesmos NCMs já usados),
com fix de duplicação/truncamento que já vinha da fonte.

Novo Dados_Financeiros_CNAE_2451_2452_2024_SerieNova.csv: primeira vez
com o financeiro aberto por classe (2451 x 2452) em vez de só o grupo
combinado 24.5 — nova tabela na seção Financeiro (só 2024).

Ainda pendente: Comex_Exportacao_Importacao_2451/2452.csv reprocessado
por NCM, e as versões "nova série IBGE" (tabelas 10451/10454) do
financeiro de Metalurgia/Fundição — arquivos ainda não chegaram.
</commit_message>
<xml_diff>
--- a/data/downloads/Financeiro.xlsx
+++ b/data/downloads/Financeiro.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Metalurgia 24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Fundicao 24.5" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2451 x 2452 (2024)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1231,7 +1232,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Fonte: IBGE/PIA-Empresa, 2007-2023.</t>
+          <t>Fonte: IBGE/PIA-Empresa, 2007-2024.</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2023,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Reúne 2451+2452 sem abertura entre eles. Fonte: IBGE/PIA-Empresa, 2007-2023.</t>
+          <t>Reúne 2451+2452 sem abertura entre eles. Fonte: IBGE/PIA-Empresa, 2007-2024.</t>
         </is>
       </c>
     </row>
@@ -2032,4 +2033,163 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Financeiro — Ferro e aço (2451) x Não ferrosos (2452)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>cnae_subclasse</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>numero_empresas_estrato_certo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>pessoal_ocupado</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>custos_despesas_totais</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>gastos_pessoal_total</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>receita_liquida_total</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>custos_operacoes_industriais</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>vbpi</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>vti</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2451</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>149</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>18427</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>6419569</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>1554424</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>6800719</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>3341793</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>6636504</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>3294711</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2452</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5168</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>3587935</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>389657</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>3408328</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>2522751</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>3414732</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>891981</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Só 2024 — primeira vez com essa abertura por classe. Fonte: IBGE/PIA-Empresa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:J7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>